<commit_message>
Fase 2: modelo de priorización, lectura de Excel y pruebas
- sitio/js/modelo.js: puntaje 0-100 por suma ponderada, reglas duras como prioridad mínima, ejes de la matriz
- sitio/js/lectura.js: lectura y validación de las hojas con mensajes claros
- criterios.xlsx: nueva hoja Escalas (tablas de conversión editables)
- generar_datos.py: fechas internas fijas para archivos idénticos en cada corrida
- pruebas/: 31 pruebas con node --test
- docs/modelo.md con dos ejemplos calculados a mano

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KVSpEyUjYEy373J9AvicYq
</commit_message>
<xml_diff>
--- a/datos/criterios.xlsx
+++ b/datos/criterios.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pesos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Umbrales" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reglas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acerca de" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escalas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Umbrales" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reglas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acerca de" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +433,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
@@ -467,7 +468,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gravedad técnica de la falla, de 1 (menor) a 4 (mayor).</t>
+          <t>Gravedad técnica de la falla, de 1 (menor) a 4 (mayor). Se convierte a 0–1 con la hoja Escalas.</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -487,7 +488,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cuántos usuarios se quedan sin servicio o con servicio deficiente (estimado).</t>
+          <t>Usuarios sin servicio o con servicio deficiente (estimado). Se convierte a 0–1 por tramos con la hoja Escalas.</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -507,7 +508,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Horas abiertas comparadas con el plazo de atención; crece al acercarse o pasar el plazo.</t>
+          <t>Qué parte del plazo de atención ya se consumió: horas abiertas ÷ plazo, con tope en 1 (vencido = 1).</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -527,7 +528,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Reportes previos en la misma localidad en los últimos 30 días.</t>
+          <t>Reportes previos en la misma localidad en los últimos 30 días. Se convierte a 0–1 con la hoja Escalas.</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -547,7 +548,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Si el reporte indica riesgo para personas o bienes.</t>
+          <t>Vale 1 si el reporte indica riesgo para personas o bienes y 0 si no.</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -560,11 +561,252 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista." type="list">
+      <formula1>"Impacto,Urgencia,Ninguno"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Criterio</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>A partir de</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Severidad</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Severidad</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Severidad</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Severidad</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Usuarios afectados</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Usuarios afectados</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Usuarios afectados</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>11</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Usuarios afectados</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>101</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Usuarios afectados</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>501</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Recurrencia</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Recurrencia</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Recurrencia</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Recurrencia</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Recurrencia</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Recurrencia</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista." type="list">
+      <formula1>"Severidad,Usuarios afectados,Recurrencia"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -660,7 +902,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -849,13 +1091,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -894,53 +1136,65 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cuánto aporta cada criterio al puntaje. Se recomienda que sumen 100.</t>
+          <t>Cuánto aporta cada criterio al puntaje (se recomienda que sumen 100) y en qué eje de la matriz cuenta.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Umbrales</t>
+          <t>Escalas</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Puntaje mínimo para cada prioridad.</t>
+          <t>Cómo se convierte cada dato a un valor de 0 a 1. Cada tramo vale desde "A partir de" hasta el inicio del siguiente.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Reglas</t>
+          <t>Umbrales</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Reglas duras: el puntaje nunca puede dejar un reporte por debajo de la prioridad mínima indicada.</t>
+          <t>Puntaje mínimo para cada prioridad.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Generado con</t>
+          <t>Reglas</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>scripts/generar_datos.py (semilla fija 20261020)</t>
+          <t>Reglas duras: el puntaje nunca puede dejar un reporte por debajo de la prioridad mínima indicada.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Generado con</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>scripts/generar_datos.py (semilla fija 20261020)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Documentación</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>docs/datos.md</t>
         </is>

</xml_diff>